<commit_message>
docs(docs): record the first dogfood run that governed a ql-pipeline pull request with its own engine
Run 35731658929 on #45: resolve announced the branch, both checkouts in every
job fetched it, and the govern job escalated on R4 as a workflow change must.
TASK051-11 closes on that evidence; TASK051-12 waits for a pull request whose
engine differs from main.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugfixes/051-dogfood-runs-main-not-the-pr/testing-plan.xlsx
+++ b/docs/bugfixes/051-dogfood-runs-main-not-the-pr/testing-plan.xlsx
@@ -997,12 +997,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>Run 35731658929 on #45: resolve annotated 'ql-pipeline governs itself: running 0xb1te/ql-pipeline@bugfixes/051-dogfood-runs-main-not-the-pr, not ql-pipeline-ref.' and the test job's second checkout fetched refs/heads/bugfixes/051-dogfood-runs-main-not-the-pr, where every earlier run fetched main</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">

</xml_diff>